<commit_message>
Commit current sensor and wiki updates
</commit_message>
<xml_diff>
--- a/project_todos.xlsx
+++ b/project_todos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jpl365prod-my.sharepoint.com/personal/mark_a_lindeman_jpl_nasa_gov/Documents/Documents/neutrino/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jpl365prod-my.sharepoint.com/personal/mark_a_lindeman_jpl_nasa_gov/Documents/Documents/neutrino/neutrino-complex-abs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_CA4A7C87D34854CF6A373CB44B1BC67F24E9EF60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4A1E7D1-7441-48D0-87F1-0B7F441E74E1}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_CA4A7C87D34854CF6A373CB44B1BC67F24E9EF60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62148A72-032E-4A5E-AEE8-43F2CCF49856}"/>
   <bookViews>
-    <workbookView xWindow="61065" yWindow="3000" windowWidth="17370" windowHeight="9795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5655" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TODOs" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -71,13 +71,19 @@
   </si>
   <si>
     <t>Correct phonn noise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">placing the heater on the KID island constrain the G somewhat because the cooling power must match the peak cooling power, </t>
+  </si>
+  <si>
+    <t>consider a second feedback KID to loosen constraints on the design</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +96,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -106,7 +120,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -114,15 +128,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,17 +459,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="110" customWidth="1"/>
+    <col min="3" max="3" width="125.44140625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="44" customWidth="1"/>
+    <col min="9" max="9" width="96" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -467,36 +501,109 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
+      <c r="C3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>